<commit_message>
🤖 Zapis ocen z www do Piwa.xlsx
</commit_message>
<xml_diff>
--- a/Piwa.xlsx
+++ b/Piwa.xlsx
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>2</v>
+        <v>2.67</v>
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Dawid: 3; Jastrząb: 1</t>
+          <t>Dawid: 3; Jastrząb: 1; Rafał: 4</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>5</v>
+        <v>3.12</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Medzz: 5</t>
+          <t>Jastrząb: 1,25; Medzz: 5</t>
         </is>
       </c>
     </row>
@@ -1683,51 +1683,293 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1">
-        <f>IF(ISBLANK(B30),"",ROW(B30)-1)</f>
-        <v/>
+      <c r="A30" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Inne Beczki</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Walloon</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Belgian IPA</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>dodane przez: Jastrząb</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Rafał: Kwasior (9.10.2026)</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Jastrząb: 2; Koma: 3,75; Rafał: 3,5</t>
+        </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1">
-        <f>IF(ISBLANK(B31),"",ROW(B31)-1)</f>
-        <v/>
+      <c r="A31" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Trzech Kumpli</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Califia</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>7</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>West Coast India Pale Ale</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>dodane przez: Jastrząb</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Jastrząb: 3; Koma: 3; Szymon: 3</t>
+        </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1">
-        <f>IF(ISBLANK(B32),"",ROW(B32)-1)</f>
-        <v/>
+      <c r="A32" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Ksiażęce złote pszeniczne</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Ksiażęce złote pszeniczne</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Inne</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>5</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>dodane przez: MlodyD</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>MlodyD: 5</t>
+        </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1">
-        <f>IF(ISBLANK(B33),"",ROW(B33)-1)</f>
-        <v/>
+      <c r="A33" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Funky Fluid</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Seychelles</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Mango NEIPA</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>dodane przez: Jastrząb</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Jastrząb: 1,25; Koma: 2,25</t>
+        </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1">
-        <f>IF(ISBLANK(B34),"",ROW(B34)-1)</f>
-        <v/>
+      <c r="A34" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Cztery ściany</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Sorbet</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Double Fruited Imperial Gose</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>dodane przez: Jastrząb</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Jastrząb: Zapach tragiczny ale smak złożony (9.10.2026)</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Jastrząb: 3,5; Koma: 1,25</t>
+        </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1">
-        <f>IF(ISBLANK(B35),"",ROW(B35)-1)</f>
-        <v/>
+      <c r="A35" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Funky Fluid</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Double Peacharine</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Double NEIPA</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>dodane przez: Jastrząb</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Koma: 2,5</t>
+        </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1">
-        <f>IF(ISBLANK(B36),"",ROW(B36)-1)</f>
-        <v/>
+      <c r="A36" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Nepo</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>One More IPA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Session IPA</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>3</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>dodane przez: Jastrząb</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Koma: 3</t>
+        </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1">
-        <f>IF(ISBLANK(B37),"",ROW(B37)-1)</f>
-        <v/>
+      <c r="A37" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Nepo</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Furious Green</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>West Coast IPA</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>dodane przez: Jastrząb</t>
+        </is>
       </c>
     </row>
     <row r="38">

</xml_diff>